<commit_message>
Add mentorship testimonials, google drive image support for cases and ui enhancements
</commit_message>
<xml_diff>
--- a/Humanitarians_Public_Impact_Stats.xlsx
+++ b/Humanitarians_Public_Impact_Stats.xlsx
@@ -2,19 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R06d0e3b5d0c04bb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonthlyStats" sheetId="2" r:id="R768829597a7c4ac7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SupportTypes" sheetId="3" r:id="R65b4fc8c857d4723"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ImpactSummary" sheetId="4" r:id="Ra1e110663c2e4a74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LastUpdated" sheetId="5" r:id="R8108c480c5ab4fe7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="6" r:id="R56b8a4107ac14c17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CaseStorySeeds" sheetId="7" r:id="R7b20c7eefe4945a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CampaignStats" sheetId="8" r:id="R28e17fe571584e0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RecipientProductSummary" sheetId="9" r:id="R68cc672e70d9497e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DataQualityNotes" sheetId="10" r:id="R730862ceb1474b5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SourceTabsAudit" sheetId="11" r:id="R720cdfba74f542f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WebsiteConfig" sheetId="12" r:id="R3e65e94bf3804946"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="13" r:id="Rb1fab46e1a814fce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re8f9eaa5e3684053"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonthlyStats" sheetId="2" r:id="Rb25f2fafa7594c4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SupportTypes" sheetId="3" r:id="Ra7cce37dfa01409a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ImpactSummary" sheetId="4" r:id="Rd73c24da7a664410"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LastUpdated" sheetId="5" r:id="R6c284d35a4224768"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="6" r:id="R0c86c3074a1341c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CaseStorySeeds" sheetId="7" r:id="R4ced355efec7449a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CampaignStats" sheetId="8" r:id="R25d04eaa589740e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RecipientProductSummary" sheetId="9" r:id="R1f242f72df3e4426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DataQualityNotes" sheetId="10" r:id="R29f080d95f4e4af6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SourceTabsAudit" sheetId="11" r:id="Rbb5c196719954381"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WebsiteConfig" sheetId="12" r:id="Rd9e1c261e28c4b19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="13" r:id="Ra2f06634e7ec4661"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MentorshipTestimonials" sheetId="14" r:id="R5553a84abeda45cf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -58,7 +59,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -80,6 +81,16 @@
         <x:fgColor rgb="0F766E"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="F8F1E7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -88,7 +99,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="38">
+  <x:cellXfs count="48">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -169,6 +180,26 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -483,7 +514,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1d2bb61c72554662"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3a189439701045e4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -513,7 +544,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc240bf7aac644714"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcf40a91a1e074565"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -581,6 +612,31 @@
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="section"/>
     <x:tableColumn id="2" name="details"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="MentorshipTestimonialsTable" displayName="MentorshipTestimonialsTable" ref="A1:Q11" headerRowCount="1">
+  <x:tableColumns count="17">
+    <x:tableColumn id="1" name="testimonial_id"/>
+    <x:tableColumn id="2" name="display_order"/>
+    <x:tableColumn id="3" name="anonymized_name"/>
+    <x:tableColumn id="4" name="public_role"/>
+    <x:tableColumn id="5" name="mentorship_track"/>
+    <x:tableColumn id="6" name="mentee_stage"/>
+    <x:tableColumn id="7" name="public_location"/>
+    <x:tableColumn id="8" name="period_label"/>
+    <x:tableColumn id="9" name="outcome_summary"/>
+    <x:tableColumn id="10" name="testimonial_text"/>
+    <x:tableColumn id="11" name="profile_image_url"/>
+    <x:tableColumn id="12" name="profile_image_alt"/>
+    <x:tableColumn id="13" name="carousel_tagline"/>
+    <x:tableColumn id="14" name="consent_received"/>
+    <x:tableColumn id="15" name="publish_status"/>
+    <x:tableColumn id="16" name="privacy_note"/>
+    <x:tableColumn id="17" name="editing_note"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </x:table>
@@ -1441,7 +1497,7 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R905802e96bf043bf"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52bcb364db9640aa"/>
 </x:worksheet>
 </file>
 
@@ -1449,153 +1505,153 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="72" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="72" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="22" t="str">
-        <x:v>note_id</x:v>
-      </x:c>
-      <x:c r="B1" s="22" t="str">
-        <x:v>severity</x:v>
-      </x:c>
-      <x:c r="C1" s="22" t="str">
+      <x:c r="A1" s="43" t="str">
         <x:v>area</x:v>
       </x:c>
-      <x:c r="D1" s="22" t="str">
-        <x:v>note</x:v>
-      </x:c>
-      <x:c r="E1" s="22" t="str">
-        <x:v>recommended_action</x:v>
+      <x:c r="B1" s="43" t="str">
+        <x:v>issue_or_decision</x:v>
+      </x:c>
+      <x:c r="C1" s="43" t="str">
+        <x:v>recommendation</x:v>
+      </x:c>
+      <x:c r="D1" s="43" t="str">
+        <x:v>public_risk</x:v>
+      </x:c>
+      <x:c r="E1" s="43" t="str">
+        <x:v>status</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="30" t="str">
-        <x:v>DQ-001</x:v>
-      </x:c>
-      <x:c r="B2" s="30" t="str">
+      <x:c r="A2" s="47" t="str">
+        <x:v>May-26 tab</x:v>
+      </x:c>
+      <x:c r="B2" s="47" t="str">
+        <x:v>May-26 appeared duplicative of Apr-26 in the source workbook.</x:v>
+      </x:c>
+      <x:c r="C2" s="47" t="str">
+        <x:v>Confirm before including in public totals.</x:v>
+      </x:c>
+      <x:c r="D2" s="47" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E2" s="47" t="str">
+        <x:v>Review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="47" t="str">
+        <x:v>Zakat_Feb_2026</x:v>
+      </x:c>
+      <x:c r="B3" s="47" t="str">
+        <x:v>Treated as consolidated Dec 2025-Apr 2026 classification data because exact month split was not fully available.</x:v>
+      </x:c>
+      <x:c r="C3" s="47" t="str">
+        <x:v>Keep consolidated label unless month-level verification is done.</x:v>
+      </x:c>
+      <x:c r="D3" s="47" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="E3" s="47" t="str">
+        <x:v>Published as consolidated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="47" t="str">
+        <x:v>Case stories</x:v>
+      </x:c>
+      <x:c r="B4" s="47" t="str">
+        <x:v>Story seeds are anonymized and draft-only until follow-up is verified.</x:v>
+      </x:c>
+      <x:c r="C4" s="47" t="str">
+        <x:v>Publish only after verification and privacy review.</x:v>
+      </x:c>
+      <x:c r="D4" s="47" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E4" s="47" t="str">
+        <x:v>Draft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="47" t="str">
+        <x:v>Case story images</x:v>
+      </x:c>
+      <x:c r="B5" s="47" t="str">
+        <x:v>Image URL columns added for three-image carousels.</x:v>
+      </x:c>
+      <x:c r="C5" s="47" t="str">
+        <x:v>Use only public Drive URLs and only after consent. Avoid identifiable faces/locations unless explicit consent exists.</x:v>
+      </x:c>
+      <x:c r="D5" s="47" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="C2" s="30" t="str">
-        <x:v>Privacy</x:v>
-      </x:c>
-      <x:c r="D2" s="30" t="str">
-        <x:v>The original Recipients List tab contains recipient names, Aadhaar numbers and addresses.</x:v>
-      </x:c>
-      <x:c r="E2" s="30" t="str">
-        <x:v>Do not publish the raw tab. Use only anonymized summaries and city/state-level locations.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="30" t="str">
-        <x:v>DQ-002</x:v>
-      </x:c>
-      <x:c r="B3" s="30" t="str">
+      <x:c r="E5" s="47" t="str">
+        <x:v>New</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="47" t="str">
+        <x:v>Mentorship testimonials</x:v>
+      </x:c>
+      <x:c r="B6" s="47" t="str">
+        <x:v>Ten editable testimonial seed rows added.</x:v>
+      </x:c>
+      <x:c r="C6" s="47" t="str">
+        <x:v>Replace placeholders with real consented quotes; frontend should render only consent_received=Yes and publish_status=Publish.</x:v>
+      </x:c>
+      <x:c r="D6" s="47" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="C3" s="30" t="str">
-        <x:v>Privacy</x:v>
-      </x:c>
-      <x:c r="D3" s="30" t="str">
-        <x:v>The Payment ID of Contributors tab contains UPI IDs and payment identifiers.</x:v>
-      </x:c>
-      <x:c r="E3" s="30" t="str">
-        <x:v>Do not publish or connect this tab to the website.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="30" t="str">
-        <x:v>DQ-003</x:v>
-      </x:c>
-      <x:c r="B4" s="30" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="C4" s="30" t="str">
-        <x:v>May-26</x:v>
-      </x:c>
-      <x:c r="D4" s="30" t="str">
-        <x:v>The May-26 tab appears to duplicate Apr-26 values and support rows.</x:v>
-      </x:c>
-      <x:c r="E4" s="30" t="str">
-        <x:v>Confirm May 2026 data before adding it to public stats.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="30" t="str">
-        <x:v>DQ-004</x:v>
-      </x:c>
-      <x:c r="B5" s="30" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="C5" s="30" t="str">
-        <x:v>Zakat_Feb_2026</x:v>
-      </x:c>
-      <x:c r="D5" s="30" t="str">
-        <x:v>The Zakat_Feb_2026 tab is a consolidated eligibility/case sheet for Dec 2025-Apr 2026; exact months are not available for all rows.</x:v>
-      </x:c>
-      <x:c r="E5" s="30" t="str">
-        <x:v>Keep consolidated label or add month-level dates in future public stats.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="30" t="str">
-        <x:v>DQ-005</x:v>
-      </x:c>
-      <x:c r="B6" s="30" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="C6" s="30" t="str">
-        <x:v>Case classification</x:v>
-      </x:c>
-      <x:c r="D6" s="30" t="str">
-        <x:v>Support categories are inferred from case descriptions using keywords.</x:v>
-      </x:c>
-      <x:c r="E6" s="30" t="str">
-        <x:v>Review category/fund-type classifications before public launch.</x:v>
+      <x:c r="E6" s="47" t="str">
+        <x:v>New</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="30" t="str">
-        <x:v>DQ-006</x:v>
-      </x:c>
-      <x:c r="B7" s="30" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="C7" s="30" t="str">
-        <x:v>Jan-2026</x:v>
-      </x:c>
-      <x:c r="D7" s="30" t="str">
-        <x:v>The source has a ₹1,014 row labelled only 'Vyapar'.</x:v>
-      </x:c>
-      <x:c r="E7" s="30" t="str">
-        <x:v>Clarify whether this is a case, bank/app fee, vendor payment, or adjustment before publishing.</x:v>
+      <x:c r="A7" s="47" t="str">
+        <x:v>RecipientProductSummary</x:v>
+      </x:c>
+      <x:c r="B7" s="47" t="str">
+        <x:v>Public tab contains aggregate product/support summaries only.</x:v>
+      </x:c>
+      <x:c r="C7" s="47" t="str">
+        <x:v>Do not publish raw Recipients List or private IDs.</x:v>
+      </x:c>
+      <x:c r="D7" s="47" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E7" s="47" t="str">
+        <x:v>Safe aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="30" t="str">
-        <x:v>DQ-007</x:v>
-      </x:c>
-      <x:c r="B8" s="30" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="C8" s="30" t="str">
-        <x:v>Mentorship stats</x:v>
-      </x:c>
-      <x:c r="D8" s="30" t="str">
-        <x:v>The workbook does not contain structured mentorship outcomes or job placement data.</x:v>
-      </x:c>
-      <x:c r="E8" s="30" t="str">
-        <x:v>Add a separate public MentorshipStats tab later with anonymized counts only.</x:v>
+      <x:c r="A8" s="47" t="str">
+        <x:v>Payment IDs</x:v>
+      </x:c>
+      <x:c r="B8" s="47" t="str">
+        <x:v>Payment ID of Contributors tab excluded from public workbook outputs.</x:v>
+      </x:c>
+      <x:c r="C8" s="47" t="str">
+        <x:v>Never expose payment IDs or donor names publicly.</x:v>
+      </x:c>
+      <x:c r="D8" s="47" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E8" s="47" t="str">
+        <x:v>Excluded</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd8bbd76b03b4f5d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09c3ab78ba3748a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2396,7 +2452,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra89851fe648b4f2b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f6d1594d47c4682"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2405,125 +2461,147 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="54" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="72" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="40" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="70" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="22" t="str">
+      <x:c r="A1" s="43" t="str">
         <x:v>key</x:v>
       </x:c>
-      <x:c r="B1" s="22" t="str">
+      <x:c r="B1" s="43" t="str">
         <x:v>value</x:v>
       </x:c>
-      <x:c r="C1" s="22" t="str">
+      <x:c r="C1" s="43" t="str">
         <x:v>notes</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="30" t="str">
+      <x:c r="A2" s="47" t="str">
         <x:v>recommended_google_sheet_name</x:v>
       </x:c>
-      <x:c r="B2" s="30" t="str">
+      <x:c r="B2" s="47" t="str">
         <x:v>Humanitarians_Public_Impact_Stats</x:v>
       </x:c>
-      <x:c r="C2" s="30" t="str">
-        <x:v>Upload this XLSX to Google Sheets using this workbook name.</x:v>
+      <x:c r="C2" s="47" t="str">
+        <x:v>Upload this XLSX to Google Sheets using this workbook name. Keep the existing Google Sheet name if replacing/updating.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="30" t="str">
+      <x:c r="A3" s="47" t="str">
         <x:v>monthly_stats_tab</x:v>
       </x:c>
-      <x:c r="B3" s="30" t="str">
+      <x:c r="B3" s="47" t="str">
         <x:v>MonthlyStats</x:v>
       </x:c>
-      <x:c r="C3" s="30" t="str">
+      <x:c r="C3" s="47" t="str">
         <x:v>Publish this tab as CSV for VITE_STATS_MONTHLY_CSV_URL.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="30" t="str">
+      <x:c r="A4" s="47" t="str">
         <x:v>support_types_tab</x:v>
       </x:c>
-      <x:c r="B4" s="30" t="str">
+      <x:c r="B4" s="47" t="str">
         <x:v>SupportTypes</x:v>
       </x:c>
-      <x:c r="C4" s="30" t="str">
+      <x:c r="C4" s="47" t="str">
         <x:v>Publish this tab as CSV for VITE_STATS_SUPPORT_TYPES_CSV_URL.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="30" t="str">
+      <x:c r="A5" s="47" t="str">
         <x:v>impact_summary_tab</x:v>
       </x:c>
-      <x:c r="B5" s="30" t="str">
+      <x:c r="B5" s="47" t="str">
         <x:v>ImpactSummary</x:v>
       </x:c>
-      <x:c r="C5" s="30" t="str">
+      <x:c r="C5" s="47" t="str">
         <x:v>Publish this tab as CSV for VITE_STATS_IMPACT_SUMMARY_CSV_URL.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="30" t="str">
+      <x:c r="A6" s="47" t="str">
         <x:v>last_updated_tab</x:v>
       </x:c>
-      <x:c r="B6" s="30" t="str">
+      <x:c r="B6" s="47" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
-      <x:c r="C6" s="30" t="str">
+      <x:c r="C6" s="47" t="str">
         <x:v>Publish this tab as CSV for VITE_STATS_LAST_UPDATED_CSV_URL.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="30" t="str">
+      <x:c r="A7" s="47" t="str">
         <x:v>case_story_tab</x:v>
       </x:c>
-      <x:c r="B7" s="30" t="str">
+      <x:c r="B7" s="47" t="str">
         <x:v>CaseStorySeeds</x:v>
       </x:c>
-      <x:c r="C7" s="30" t="str">
-        <x:v>Optional: publish as CSV only if you want anonymized story cards to update from Sheets.</x:v>
+      <x:c r="C7" s="47" t="str">
+        <x:v>Publish as CSV for VITE_STATS_CASE_STORIES_CSV_URL. Now includes image_url_1, image_url_2, image_url_3 for case-story carousels.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="30" t="str">
+      <x:c r="A8" s="47" t="str">
+        <x:v>mentorship_testimonials_tab</x:v>
+      </x:c>
+      <x:c r="B8" s="47" t="str">
+        <x:v>MentorshipTestimonials</x:v>
+      </x:c>
+      <x:c r="C8" s="47" t="str">
+        <x:v>Publish as CSV for VITE_STATS_MENTORSHIP_TESTIMONIALS_CSV_URL. Carousel should render only publish_status=Publish and consent_received=Yes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="47" t="str">
         <x:v>reports_tab</x:v>
       </x:c>
-      <x:c r="B8" s="30" t="str">
+      <x:c r="B9" s="47" t="str">
         <x:v>Reports</x:v>
       </x:c>
-      <x:c r="C8" s="30" t="str">
-        <x:v>Optional: publish as CSV for the transparency/report page.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="30" t="str">
+      <x:c r="C9" s="47" t="str">
+        <x:v>Optional: publish as CSV for VITE_STATS_REPORTS_CSV_URL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="47" t="str">
+        <x:v>case_story_image_columns</x:v>
+      </x:c>
+      <x:c r="B10" s="47" t="str">
+        <x:v>image_url_1,image_url_2,image_url_3</x:v>
+      </x:c>
+      <x:c r="C10" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs in these columns. Use consent/status fields before publishing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="47" t="str">
         <x:v>public_privacy_rule</x:v>
       </x:c>
-      <x:c r="B9" s="30" t="str">
+      <x:c r="B11" s="47" t="str">
         <x:v>Only aggregated/anonymized data goes public</x:v>
       </x:c>
-      <x:c r="C9" s="30" t="str">
+      <x:c r="C11" s="47" t="str">
         <x:v>Never publish raw contributor or recipient tabs.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="30" t="str">
+    <x:row r="12">
+      <x:c r="A12" s="47" t="str">
         <x:v>frontend_stack</x:v>
       </x:c>
-      <x:c r="B10" s="30" t="str">
+      <x:c r="B12" s="47" t="str">
         <x:v>React + TypeScript + Vite + Recharts + PapaParse</x:v>
       </x:c>
-      <x:c r="C10" s="30" t="str">
-        <x:v>No backend required for public stats.</x:v>
+      <x:c r="C12" s="47" t="str">
+        <x:v>No backend required for public stats and public testimonials.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R287ac8ac1f754b95"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d5f3f61ecf849a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2532,86 +2610,704 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="94" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="90" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="22" t="str">
+      <x:c r="A1" s="43" t="str">
         <x:v>section</x:v>
       </x:c>
-      <x:c r="B1" s="22" t="str">
+      <x:c r="B1" s="43" t="str">
         <x:v>details</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="30" t="str">
+      <x:c r="A2" s="47" t="str">
         <x:v>Workbook purpose</x:v>
       </x:c>
-      <x:c r="B2" s="30" t="str">
-        <x:v>Public, privacy-safe impact statistics for the Humanitarians website.</x:v>
+      <x:c r="B2" s="47" t="str">
+        <x:v>Public, privacy-safe impact statistics, case-story seeds, case-story image URLs, and mentorship testimonial seeds for the Humanitarians website.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="30" t="str">
+      <x:c r="A3" s="47" t="str">
         <x:v>Recommended Google Sheet name</x:v>
       </x:c>
-      <x:c r="B3" s="30" t="str">
+      <x:c r="B3" s="47" t="str">
         <x:v>Humanitarians_Public_Impact_Stats</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="30" t="str">
+      <x:c r="A4" s="47" t="str">
         <x:v>Main website tabs</x:v>
       </x:c>
-      <x:c r="B4" s="30" t="str">
-        <x:v>MonthlyStats, SupportTypes, ImpactSummary, LastUpdated, Reports, CaseStorySeeds.</x:v>
+      <x:c r="B4" s="47" t="str">
+        <x:v>MonthlyStats, SupportTypes, ImpactSummary, LastUpdated, Reports, CaseStorySeeds, MentorshipTestimonials.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="30" t="str">
+      <x:c r="A5" s="47" t="str">
+        <x:v>Case-story images</x:v>
+      </x:c>
+      <x:c r="B5" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs into CaseStorySeeds image_url_1, image_url_2, and image_url_3. Use image_alt and image_caption fields for accessible carousel display.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="47" t="str">
+        <x:v>Mentorship testimonials</x:v>
+      </x:c>
+      <x:c r="B6" s="47" t="str">
+        <x:v>Fill MentorshipTestimonials with real consented mentee quotes. Publish only rows with consent_received=Yes and publish_status=Publish.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="47" t="str">
         <x:v>Privacy exclusions</x:v>
       </x:c>
-      <x:c r="B5" s="30" t="str">
-        <x:v>Raw recipient names, Aadhaar numbers, addresses, contributor names and UPI IDs are not copied into public stats.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="30" t="str">
+      <x:c r="B7" s="47" t="str">
+        <x:v>Raw recipient names, Aadhaar numbers, addresses, contributor names, UPI IDs, payment IDs, private notes, and private documents are not copied into public stats.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="47" t="str">
         <x:v>Upload flow</x:v>
       </x:c>
-      <x:c r="B6" s="30" t="str">
+      <x:c r="B8" s="47" t="str">
         <x:v>Upload this XLSX to Google Sheets, check each tab, then publish individual website tabs to CSV.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="30" t="str">
+    <x:row r="9">
+      <x:c r="A9" s="47" t="str">
         <x:v>CSV publishing</x:v>
       </x:c>
-      <x:c r="B7" s="30" t="str">
+      <x:c r="B9" s="47" t="str">
         <x:v>In Google Sheets: File &gt; Share &gt; Publish to web &gt; choose a tab &gt; CSV. Paste each CSV URL into the React .env file.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="30" t="str">
+    <x:row r="10">
+      <x:c r="A10" s="47" t="str">
         <x:v>Before launch</x:v>
       </x:c>
-      <x:c r="B8" s="30" t="str">
-        <x:v>Review DataQualityNotes and verify May-26, Zakat_Feb_2026 consolidated period, and any story candidates.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="30" t="str">
+      <x:c r="B10" s="47" t="str">
+        <x:v>Review DataQualityNotes and verify any story/testimonial candidates. Do not publish placeholders as real quotes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="47" t="str">
         <x:v>Website rule</x:v>
       </x:c>
-      <x:c r="B9" s="30" t="str">
+      <x:c r="B11" s="47" t="str">
         <x:v>Frontend may fetch public CSVs directly. This is safe only because these tabs contain no private data.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37abd4e5d6ab4c70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R312c98cc03694db7"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="42" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="36" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="36" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="24" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="42" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="42" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="43" t="str">
+        <x:v>testimonial_id</x:v>
+      </x:c>
+      <x:c r="B1" s="43" t="str">
+        <x:v>display_order</x:v>
+      </x:c>
+      <x:c r="C1" s="43" t="str">
+        <x:v>anonymized_name</x:v>
+      </x:c>
+      <x:c r="D1" s="43" t="str">
+        <x:v>public_role</x:v>
+      </x:c>
+      <x:c r="E1" s="43" t="str">
+        <x:v>mentorship_track</x:v>
+      </x:c>
+      <x:c r="F1" s="43" t="str">
+        <x:v>mentee_stage</x:v>
+      </x:c>
+      <x:c r="G1" s="43" t="str">
+        <x:v>public_location</x:v>
+      </x:c>
+      <x:c r="H1" s="43" t="str">
+        <x:v>period_label</x:v>
+      </x:c>
+      <x:c r="I1" s="43" t="str">
+        <x:v>outcome_summary</x:v>
+      </x:c>
+      <x:c r="J1" s="43" t="str">
+        <x:v>testimonial_text</x:v>
+      </x:c>
+      <x:c r="K1" s="43" t="str">
+        <x:v>profile_image_url</x:v>
+      </x:c>
+      <x:c r="L1" s="43" t="str">
+        <x:v>profile_image_alt</x:v>
+      </x:c>
+      <x:c r="M1" s="43" t="str">
+        <x:v>carousel_tagline</x:v>
+      </x:c>
+      <x:c r="N1" s="43" t="str">
+        <x:v>consent_received</x:v>
+      </x:c>
+      <x:c r="O1" s="43" t="str">
+        <x:v>publish_status</x:v>
+      </x:c>
+      <x:c r="P1" s="43" t="str">
+        <x:v>privacy_note</x:v>
+      </x:c>
+      <x:c r="Q1" s="43" t="str">
+        <x:v>editing_note</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="47" t="str">
+        <x:v>HUM-MENT-001</x:v>
+      </x:c>
+      <x:c r="B2" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C2" s="47" t="str">
+        <x:v>Anonymized mentee 1</x:v>
+      </x:c>
+      <x:c r="D2" s="47" t="str">
+        <x:v>Mentee</x:v>
+      </x:c>
+      <x:c r="E2" s="47" t="str">
+        <x:v>Resume Review</x:v>
+      </x:c>
+      <x:c r="F2" s="47" t="str">
+        <x:v>Final-year student</x:v>
+      </x:c>
+      <x:c r="G2" s="47" t="str">
+        <x:v>Public-safe city/state only</x:v>
+      </x:c>
+      <x:c r="H2" s="47" t="str">
+        <x:v>Add month/year</x:v>
+      </x:c>
+      <x:c r="I2" s="47" t="str">
+        <x:v>Add only a verified outcome, e.g. resume improved, interview prepared, offer received, internship secured, or course completed.</x:v>
+      </x:c>
+      <x:c r="J2" s="47" t="str">
+        <x:v>Replace this placeholder with a real mentee testimonial after consent. Do not publish this placeholder as a real quote.</x:v>
+      </x:c>
+      <x:c r="K2" s="47" t="str"/>
+      <x:c r="L2" s="47" t="str">
+        <x:v>Optional anonymized profile image/avatar for HUM-MENT-001; add only after consent.</x:v>
+      </x:c>
+      <x:c r="M2" s="47" t="str">
+        <x:v>Resume clarity</x:v>
+      </x:c>
+      <x:c r="N2" s="47" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="O2" s="47" t="str">
+        <x:v>Draft - replace with real consented testimonial</x:v>
+      </x:c>
+      <x:c r="P2" s="47" t="str">
+        <x:v>Anonymized public testimonial; no full name, phone, address, ID, private documents, employer-sensitive details, or donor identity included.</x:v>
+      </x:c>
+      <x:c r="Q2" s="47" t="str">
+        <x:v>When ready: add real quote, verify outcome, set consent_received=Yes, set publish_status=Publish.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="47" t="str">
+        <x:v>HUM-MENT-002</x:v>
+      </x:c>
+      <x:c r="B3" s="47" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C3" s="47" t="str">
+        <x:v>Anonymized mentee 2</x:v>
+      </x:c>
+      <x:c r="D3" s="47" t="str">
+        <x:v>Mentee</x:v>
+      </x:c>
+      <x:c r="E3" s="47" t="str">
+        <x:v>Interview Preparation</x:v>
+      </x:c>
+      <x:c r="F3" s="47" t="str">
+        <x:v>Graduate job seeker</x:v>
+      </x:c>
+      <x:c r="G3" s="47" t="str">
+        <x:v>Public-safe city/state only</x:v>
+      </x:c>
+      <x:c r="H3" s="47" t="str">
+        <x:v>Add month/year</x:v>
+      </x:c>
+      <x:c r="I3" s="47" t="str">
+        <x:v>Add only a verified outcome, e.g. resume improved, interview prepared, offer received, internship secured, or course completed.</x:v>
+      </x:c>
+      <x:c r="J3" s="47" t="str">
+        <x:v>Replace this placeholder with a real mentee testimonial after consent. Do not publish this placeholder as a real quote.</x:v>
+      </x:c>
+      <x:c r="K3" s="47" t="str"/>
+      <x:c r="L3" s="47" t="str">
+        <x:v>Optional anonymized profile image/avatar for HUM-MENT-002; add only after consent.</x:v>
+      </x:c>
+      <x:c r="M3" s="47" t="str">
+        <x:v>Interview confidence</x:v>
+      </x:c>
+      <x:c r="N3" s="47" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="O3" s="47" t="str">
+        <x:v>Draft - replace with real consented testimonial</x:v>
+      </x:c>
+      <x:c r="P3" s="47" t="str">
+        <x:v>Anonymized public testimonial; no full name, phone, address, ID, private documents, employer-sensitive details, or donor identity included.</x:v>
+      </x:c>
+      <x:c r="Q3" s="47" t="str">
+        <x:v>When ready: add real quote, verify outcome, set consent_received=Yes, set publish_status=Publish.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="47" t="str">
+        <x:v>HUM-MENT-003</x:v>
+      </x:c>
+      <x:c r="B4" s="47" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C4" s="47" t="str">
+        <x:v>Anonymized mentee 3</x:v>
+      </x:c>
+      <x:c r="D4" s="47" t="str">
+        <x:v>Mentee</x:v>
+      </x:c>
+      <x:c r="E4" s="47" t="str">
+        <x:v>Coding / IT Guidance</x:v>
+      </x:c>
+      <x:c r="F4" s="47" t="str">
+        <x:v>Early-career learner</x:v>
+      </x:c>
+      <x:c r="G4" s="47" t="str">
+        <x:v>Public-safe city/state only</x:v>
+      </x:c>
+      <x:c r="H4" s="47" t="str">
+        <x:v>Add month/year</x:v>
+      </x:c>
+      <x:c r="I4" s="47" t="str">
+        <x:v>Add only a verified outcome, e.g. resume improved, interview prepared, offer received, internship secured, or course completed.</x:v>
+      </x:c>
+      <x:c r="J4" s="47" t="str">
+        <x:v>Replace this placeholder with a real mentee testimonial after consent. Do not publish this placeholder as a real quote.</x:v>
+      </x:c>
+      <x:c r="K4" s="47" t="str"/>
+      <x:c r="L4" s="47" t="str">
+        <x:v>Optional anonymized profile image/avatar for HUM-MENT-003; add only after consent.</x:v>
+      </x:c>
+      <x:c r="M4" s="47" t="str">
+        <x:v>Guided practice</x:v>
+      </x:c>
+      <x:c r="N4" s="47" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="O4" s="47" t="str">
+        <x:v>Draft - replace with real consented testimonial</x:v>
+      </x:c>
+      <x:c r="P4" s="47" t="str">
+        <x:v>Anonymized public testimonial; no full name, phone, address, ID, private documents, employer-sensitive details, or donor identity included.</x:v>
+      </x:c>
+      <x:c r="Q4" s="47" t="str">
+        <x:v>When ready: add real quote, verify outcome, set consent_received=Yes, set publish_status=Publish.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="47" t="str">
+        <x:v>HUM-MENT-004</x:v>
+      </x:c>
+      <x:c r="B5" s="47" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C5" s="47" t="str">
+        <x:v>Anonymized mentee 4</x:v>
+      </x:c>
+      <x:c r="D5" s="47" t="str">
+        <x:v>Mentee</x:v>
+      </x:c>
+      <x:c r="E5" s="47" t="str">
+        <x:v>Data / Analytics Guidance</x:v>
+      </x:c>
+      <x:c r="F5" s="47" t="str">
+        <x:v>Graduate job seeker</x:v>
+      </x:c>
+      <x:c r="G5" s="47" t="str">
+        <x:v>Public-safe city/state only</x:v>
+      </x:c>
+      <x:c r="H5" s="47" t="str">
+        <x:v>Add month/year</x:v>
+      </x:c>
+      <x:c r="I5" s="47" t="str">
+        <x:v>Add only a verified outcome, e.g. resume improved, interview prepared, offer received, internship secured, or course completed.</x:v>
+      </x:c>
+      <x:c r="J5" s="47" t="str">
+        <x:v>Replace this placeholder with a real mentee testimonial after consent. Do not publish this placeholder as a real quote.</x:v>
+      </x:c>
+      <x:c r="K5" s="47" t="str"/>
+      <x:c r="L5" s="47" t="str">
+        <x:v>Optional anonymized profile image/avatar for HUM-MENT-004; add only after consent.</x:v>
+      </x:c>
+      <x:c r="M5" s="47" t="str">
+        <x:v>Skill direction</x:v>
+      </x:c>
+      <x:c r="N5" s="47" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="O5" s="47" t="str">
+        <x:v>Draft - replace with real consented testimonial</x:v>
+      </x:c>
+      <x:c r="P5" s="47" t="str">
+        <x:v>Anonymized public testimonial; no full name, phone, address, ID, private documents, employer-sensitive details, or donor identity included.</x:v>
+      </x:c>
+      <x:c r="Q5" s="47" t="str">
+        <x:v>When ready: add real quote, verify outcome, set consent_received=Yes, set publish_status=Publish.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="47" t="str">
+        <x:v>HUM-MENT-005</x:v>
+      </x:c>
+      <x:c r="B6" s="47" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C6" s="47" t="str">
+        <x:v>Anonymized mentee 5</x:v>
+      </x:c>
+      <x:c r="D6" s="47" t="str">
+        <x:v>Mentee</x:v>
+      </x:c>
+      <x:c r="E6" s="47" t="str">
+        <x:v>Course Selection</x:v>
+      </x:c>
+      <x:c r="F6" s="47" t="str">
+        <x:v>Undergraduate student</x:v>
+      </x:c>
+      <x:c r="G6" s="47" t="str">
+        <x:v>Public-safe city/state only</x:v>
+      </x:c>
+      <x:c r="H6" s="47" t="str">
+        <x:v>Add month/year</x:v>
+      </x:c>
+      <x:c r="I6" s="47" t="str">
+        <x:v>Add only a verified outcome, e.g. resume improved, interview prepared, offer received, internship secured, or course completed.</x:v>
+      </x:c>
+      <x:c r="J6" s="47" t="str">
+        <x:v>Replace this placeholder with a real mentee testimonial after consent. Do not publish this placeholder as a real quote.</x:v>
+      </x:c>
+      <x:c r="K6" s="47" t="str"/>
+      <x:c r="L6" s="47" t="str">
+        <x:v>Optional anonymized profile image/avatar for HUM-MENT-005; add only after consent.</x:v>
+      </x:c>
+      <x:c r="M6" s="47" t="str">
+        <x:v>Course clarity</x:v>
+      </x:c>
+      <x:c r="N6" s="47" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="O6" s="47" t="str">
+        <x:v>Draft - replace with real consented testimonial</x:v>
+      </x:c>
+      <x:c r="P6" s="47" t="str">
+        <x:v>Anonymized public testimonial; no full name, phone, address, ID, private documents, employer-sensitive details, or donor identity included.</x:v>
+      </x:c>
+      <x:c r="Q6" s="47" t="str">
+        <x:v>When ready: add real quote, verify outcome, set consent_received=Yes, set publish_status=Publish.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="47" t="str">
+        <x:v>HUM-MENT-006</x:v>
+      </x:c>
+      <x:c r="B7" s="47" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C7" s="47" t="str">
+        <x:v>Anonymized mentee 6</x:v>
+      </x:c>
+      <x:c r="D7" s="47" t="str">
+        <x:v>Mentee</x:v>
+      </x:c>
+      <x:c r="E7" s="47" t="str">
+        <x:v>English Communication</x:v>
+      </x:c>
+      <x:c r="F7" s="47" t="str">
+        <x:v>Student job seeker</x:v>
+      </x:c>
+      <x:c r="G7" s="47" t="str">
+        <x:v>Public-safe city/state only</x:v>
+      </x:c>
+      <x:c r="H7" s="47" t="str">
+        <x:v>Add month/year</x:v>
+      </x:c>
+      <x:c r="I7" s="47" t="str">
+        <x:v>Add only a verified outcome, e.g. resume improved, interview prepared, offer received, internship secured, or course completed.</x:v>
+      </x:c>
+      <x:c r="J7" s="47" t="str">
+        <x:v>Replace this placeholder with a real mentee testimonial after consent. Do not publish this placeholder as a real quote.</x:v>
+      </x:c>
+      <x:c r="K7" s="47" t="str"/>
+      <x:c r="L7" s="47" t="str">
+        <x:v>Optional anonymized profile image/avatar for HUM-MENT-006; add only after consent.</x:v>
+      </x:c>
+      <x:c r="M7" s="47" t="str">
+        <x:v>Communication support</x:v>
+      </x:c>
+      <x:c r="N7" s="47" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="O7" s="47" t="str">
+        <x:v>Draft - replace with real consented testimonial</x:v>
+      </x:c>
+      <x:c r="P7" s="47" t="str">
+        <x:v>Anonymized public testimonial; no full name, phone, address, ID, private documents, employer-sensitive details, or donor identity included.</x:v>
+      </x:c>
+      <x:c r="Q7" s="47" t="str">
+        <x:v>When ready: add real quote, verify outcome, set consent_received=Yes, set publish_status=Publish.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="47" t="str">
+        <x:v>HUM-MENT-007</x:v>
+      </x:c>
+      <x:c r="B8" s="47" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C8" s="47" t="str">
+        <x:v>Anonymized mentee 7</x:v>
+      </x:c>
+      <x:c r="D8" s="47" t="str">
+        <x:v>Mentee</x:v>
+      </x:c>
+      <x:c r="E8" s="47" t="str">
+        <x:v>Career Direction</x:v>
+      </x:c>
+      <x:c r="F8" s="47" t="str">
+        <x:v>Graduate job seeker</x:v>
+      </x:c>
+      <x:c r="G8" s="47" t="str">
+        <x:v>Public-safe city/state only</x:v>
+      </x:c>
+      <x:c r="H8" s="47" t="str">
+        <x:v>Add month/year</x:v>
+      </x:c>
+      <x:c r="I8" s="47" t="str">
+        <x:v>Add only a verified outcome, e.g. resume improved, interview prepared, offer received, internship secured, or course completed.</x:v>
+      </x:c>
+      <x:c r="J8" s="47" t="str">
+        <x:v>Replace this placeholder with a real mentee testimonial after consent. Do not publish this placeholder as a real quote.</x:v>
+      </x:c>
+      <x:c r="K8" s="47" t="str"/>
+      <x:c r="L8" s="47" t="str">
+        <x:v>Optional anonymized profile image/avatar for HUM-MENT-007; add only after consent.</x:v>
+      </x:c>
+      <x:c r="M8" s="47" t="str">
+        <x:v>Career roadmap</x:v>
+      </x:c>
+      <x:c r="N8" s="47" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="O8" s="47" t="str">
+        <x:v>Draft - replace with real consented testimonial</x:v>
+      </x:c>
+      <x:c r="P8" s="47" t="str">
+        <x:v>Anonymized public testimonial; no full name, phone, address, ID, private documents, employer-sensitive details, or donor identity included.</x:v>
+      </x:c>
+      <x:c r="Q8" s="47" t="str">
+        <x:v>When ready: add real quote, verify outcome, set consent_received=Yes, set publish_status=Publish.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="47" t="str">
+        <x:v>HUM-MENT-008</x:v>
+      </x:c>
+      <x:c r="B9" s="47" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C9" s="47" t="str">
+        <x:v>Anonymized mentee 8</x:v>
+      </x:c>
+      <x:c r="D9" s="47" t="str">
+        <x:v>Mentee</x:v>
+      </x:c>
+      <x:c r="E9" s="47" t="str">
+        <x:v>Job Search Strategy</x:v>
+      </x:c>
+      <x:c r="F9" s="47" t="str">
+        <x:v>Fresher candidate</x:v>
+      </x:c>
+      <x:c r="G9" s="47" t="str">
+        <x:v>Public-safe city/state only</x:v>
+      </x:c>
+      <x:c r="H9" s="47" t="str">
+        <x:v>Add month/year</x:v>
+      </x:c>
+      <x:c r="I9" s="47" t="str">
+        <x:v>Add only a verified outcome, e.g. resume improved, interview prepared, offer received, internship secured, or course completed.</x:v>
+      </x:c>
+      <x:c r="J9" s="47" t="str">
+        <x:v>Replace this placeholder with a real mentee testimonial after consent. Do not publish this placeholder as a real quote.</x:v>
+      </x:c>
+      <x:c r="K9" s="47" t="str"/>
+      <x:c r="L9" s="47" t="str">
+        <x:v>Optional anonymized profile image/avatar for HUM-MENT-008; add only after consent.</x:v>
+      </x:c>
+      <x:c r="M9" s="47" t="str">
+        <x:v>Search structure</x:v>
+      </x:c>
+      <x:c r="N9" s="47" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="O9" s="47" t="str">
+        <x:v>Draft - replace with real consented testimonial</x:v>
+      </x:c>
+      <x:c r="P9" s="47" t="str">
+        <x:v>Anonymized public testimonial; no full name, phone, address, ID, private documents, employer-sensitive details, or donor identity included.</x:v>
+      </x:c>
+      <x:c r="Q9" s="47" t="str">
+        <x:v>When ready: add real quote, verify outcome, set consent_received=Yes, set publish_status=Publish.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="47" t="str">
+        <x:v>HUM-MENT-009</x:v>
+      </x:c>
+      <x:c r="B10" s="47" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C10" s="47" t="str">
+        <x:v>Anonymized mentee 9</x:v>
+      </x:c>
+      <x:c r="D10" s="47" t="str">
+        <x:v>Mentee</x:v>
+      </x:c>
+      <x:c r="E10" s="47" t="str">
+        <x:v>LinkedIn / Portfolio Review</x:v>
+      </x:c>
+      <x:c r="F10" s="47" t="str">
+        <x:v>Early-career learner</x:v>
+      </x:c>
+      <x:c r="G10" s="47" t="str">
+        <x:v>Public-safe city/state only</x:v>
+      </x:c>
+      <x:c r="H10" s="47" t="str">
+        <x:v>Add month/year</x:v>
+      </x:c>
+      <x:c r="I10" s="47" t="str">
+        <x:v>Add only a verified outcome, e.g. resume improved, interview prepared, offer received, internship secured, or course completed.</x:v>
+      </x:c>
+      <x:c r="J10" s="47" t="str">
+        <x:v>Replace this placeholder with a real mentee testimonial after consent. Do not publish this placeholder as a real quote.</x:v>
+      </x:c>
+      <x:c r="K10" s="47" t="str"/>
+      <x:c r="L10" s="47" t="str">
+        <x:v>Optional anonymized profile image/avatar for HUM-MENT-009; add only after consent.</x:v>
+      </x:c>
+      <x:c r="M10" s="47" t="str">
+        <x:v>Profile polish</x:v>
+      </x:c>
+      <x:c r="N10" s="47" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="O10" s="47" t="str">
+        <x:v>Draft - replace with real consented testimonial</x:v>
+      </x:c>
+      <x:c r="P10" s="47" t="str">
+        <x:v>Anonymized public testimonial; no full name, phone, address, ID, private documents, employer-sensitive details, or donor identity included.</x:v>
+      </x:c>
+      <x:c r="Q10" s="47" t="str">
+        <x:v>When ready: add real quote, verify outcome, set consent_received=Yes, set publish_status=Publish.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="47" t="str">
+        <x:v>HUM-MENT-010</x:v>
+      </x:c>
+      <x:c r="B11" s="47" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C11" s="47" t="str">
+        <x:v>Anonymized mentee 10</x:v>
+      </x:c>
+      <x:c r="D11" s="47" t="str">
+        <x:v>Mentee</x:v>
+      </x:c>
+      <x:c r="E11" s="47" t="str">
+        <x:v>Mentorship + Course Sponsorship</x:v>
+      </x:c>
+      <x:c r="F11" s="47" t="str">
+        <x:v>Course-sponsored mentee</x:v>
+      </x:c>
+      <x:c r="G11" s="47" t="str">
+        <x:v>Public-safe city/state only</x:v>
+      </x:c>
+      <x:c r="H11" s="47" t="str">
+        <x:v>Add month/year</x:v>
+      </x:c>
+      <x:c r="I11" s="47" t="str">
+        <x:v>Add only a verified outcome, e.g. resume improved, interview prepared, offer received, internship secured, or course completed.</x:v>
+      </x:c>
+      <x:c r="J11" s="47" t="str">
+        <x:v>Replace this placeholder with a real mentee testimonial after consent. Do not publish this placeholder as a real quote.</x:v>
+      </x:c>
+      <x:c r="K11" s="47" t="str"/>
+      <x:c r="L11" s="47" t="str">
+        <x:v>Optional anonymized profile image/avatar for HUM-MENT-010; add only after consent.</x:v>
+      </x:c>
+      <x:c r="M11" s="47" t="str">
+        <x:v>Learning support</x:v>
+      </x:c>
+      <x:c r="N11" s="47" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="O11" s="47" t="str">
+        <x:v>Draft - replace with real consented testimonial</x:v>
+      </x:c>
+      <x:c r="P11" s="47" t="str">
+        <x:v>Anonymized public testimonial; no full name, phone, address, ID, private documents, employer-sensitive details, or donor identity included.</x:v>
+      </x:c>
+      <x:c r="Q11" s="47" t="str">
+        <x:v>When ready: add real quote, verify outcome, set consent_received=Yes, set publish_status=Publish.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="N2:N101">
+      <x:formula1>"Yes,No,Pending"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="O2:O101">
+      <x:formula1>"Draft - replace with real consented testimonial,Publish,Archive,Review required"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01ac113f985e4f70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4033,7 +4729,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68eb9dbe13b24ada"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4174e1a46ae498b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4307,7 +5003,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R602f25a12936476f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf649c81831c4151"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4632,7 +5328,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe6a9aa439404432"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7380a8b83a6846ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4678,7 +5374,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95f051293c974aca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cf2a0760f2a4cc7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5578,7 +6274,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38ad5355ef4e4b07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1eb7ce088d794579"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5604,6 +6300,17 @@
     <x:col min="15" max="15" width="60" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="16" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="30" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="28" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="28" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="28" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="28" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="28" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="28" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="28" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="28" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="28" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="28" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -5658,6 +6365,39 @@
       <x:c r="Q1" s="22" t="str">
         <x:v>publish_status</x:v>
       </x:c>
+      <x:c r="R1" s="43" t="str">
+        <x:v>image_url_1</x:v>
+      </x:c>
+      <x:c r="S1" s="43" t="str">
+        <x:v>image_alt_1</x:v>
+      </x:c>
+      <x:c r="T1" s="43" t="str">
+        <x:v>image_caption_1</x:v>
+      </x:c>
+      <x:c r="U1" s="43" t="str">
+        <x:v>image_url_2</x:v>
+      </x:c>
+      <x:c r="V1" s="43" t="str">
+        <x:v>image_alt_2</x:v>
+      </x:c>
+      <x:c r="W1" s="43" t="str">
+        <x:v>image_caption_2</x:v>
+      </x:c>
+      <x:c r="X1" s="43" t="str">
+        <x:v>image_url_3</x:v>
+      </x:c>
+      <x:c r="Y1" s="43" t="str">
+        <x:v>image_alt_3</x:v>
+      </x:c>
+      <x:c r="Z1" s="43" t="str">
+        <x:v>image_caption_3</x:v>
+      </x:c>
+      <x:c r="AA1" s="43" t="str">
+        <x:v>image_consent_status</x:v>
+      </x:c>
+      <x:c r="AB1" s="43" t="str">
+        <x:v>image_publish_notes</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="30" t="str">
@@ -5711,6 +6451,33 @@
       <x:c r="Q2" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R2" s="47" t="str"/>
+      <x:c r="S2" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-001</x:v>
+      </x:c>
+      <x:c r="T2" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U2" s="47" t="str"/>
+      <x:c r="V2" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-001</x:v>
+      </x:c>
+      <x:c r="W2" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X2" s="47" t="str"/>
+      <x:c r="Y2" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-001</x:v>
+      </x:c>
+      <x:c r="Z2" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA2" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB2" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="30" t="str">
@@ -5764,6 +6531,33 @@
       <x:c r="Q3" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R3" s="47" t="str"/>
+      <x:c r="S3" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-002</x:v>
+      </x:c>
+      <x:c r="T3" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U3" s="47" t="str"/>
+      <x:c r="V3" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-002</x:v>
+      </x:c>
+      <x:c r="W3" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X3" s="47" t="str"/>
+      <x:c r="Y3" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-002</x:v>
+      </x:c>
+      <x:c r="Z3" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA3" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB3" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="30" t="str">
@@ -5817,6 +6611,33 @@
       <x:c r="Q4" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R4" s="47" t="str"/>
+      <x:c r="S4" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-003</x:v>
+      </x:c>
+      <x:c r="T4" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U4" s="47" t="str"/>
+      <x:c r="V4" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-003</x:v>
+      </x:c>
+      <x:c r="W4" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X4" s="47" t="str"/>
+      <x:c r="Y4" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-003</x:v>
+      </x:c>
+      <x:c r="Z4" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA4" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB4" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="30" t="str">
@@ -5870,6 +6691,33 @@
       <x:c r="Q5" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R5" s="47" t="str"/>
+      <x:c r="S5" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-004</x:v>
+      </x:c>
+      <x:c r="T5" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U5" s="47" t="str"/>
+      <x:c r="V5" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-004</x:v>
+      </x:c>
+      <x:c r="W5" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X5" s="47" t="str"/>
+      <x:c r="Y5" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-004</x:v>
+      </x:c>
+      <x:c r="Z5" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA5" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB5" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="30" t="str">
@@ -5923,6 +6771,33 @@
       <x:c r="Q6" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R6" s="47" t="str"/>
+      <x:c r="S6" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-005</x:v>
+      </x:c>
+      <x:c r="T6" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U6" s="47" t="str"/>
+      <x:c r="V6" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-005</x:v>
+      </x:c>
+      <x:c r="W6" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X6" s="47" t="str"/>
+      <x:c r="Y6" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-005</x:v>
+      </x:c>
+      <x:c r="Z6" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA6" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB6" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="30" t="str">
@@ -5976,6 +6851,33 @@
       <x:c r="Q7" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R7" s="47" t="str"/>
+      <x:c r="S7" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-006</x:v>
+      </x:c>
+      <x:c r="T7" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U7" s="47" t="str"/>
+      <x:c r="V7" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-006</x:v>
+      </x:c>
+      <x:c r="W7" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X7" s="47" t="str"/>
+      <x:c r="Y7" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-006</x:v>
+      </x:c>
+      <x:c r="Z7" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA7" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB7" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="30" t="str">
@@ -6029,6 +6931,33 @@
       <x:c r="Q8" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R8" s="47" t="str"/>
+      <x:c r="S8" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-007</x:v>
+      </x:c>
+      <x:c r="T8" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U8" s="47" t="str"/>
+      <x:c r="V8" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-007</x:v>
+      </x:c>
+      <x:c r="W8" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X8" s="47" t="str"/>
+      <x:c r="Y8" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-007</x:v>
+      </x:c>
+      <x:c r="Z8" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA8" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB8" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="30" t="str">
@@ -6082,6 +7011,33 @@
       <x:c r="Q9" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R9" s="47" t="str"/>
+      <x:c r="S9" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-008</x:v>
+      </x:c>
+      <x:c r="T9" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U9" s="47" t="str"/>
+      <x:c r="V9" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-008</x:v>
+      </x:c>
+      <x:c r="W9" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X9" s="47" t="str"/>
+      <x:c r="Y9" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-008</x:v>
+      </x:c>
+      <x:c r="Z9" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA9" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB9" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="30" t="str">
@@ -6135,6 +7091,33 @@
       <x:c r="Q10" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R10" s="47" t="str"/>
+      <x:c r="S10" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-009</x:v>
+      </x:c>
+      <x:c r="T10" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U10" s="47" t="str"/>
+      <x:c r="V10" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-009</x:v>
+      </x:c>
+      <x:c r="W10" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X10" s="47" t="str"/>
+      <x:c r="Y10" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-009</x:v>
+      </x:c>
+      <x:c r="Z10" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA10" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB10" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="30" t="str">
@@ -6188,6 +7171,33 @@
       <x:c r="Q11" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R11" s="47" t="str"/>
+      <x:c r="S11" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-010</x:v>
+      </x:c>
+      <x:c r="T11" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U11" s="47" t="str"/>
+      <x:c r="V11" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-010</x:v>
+      </x:c>
+      <x:c r="W11" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X11" s="47" t="str"/>
+      <x:c r="Y11" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-010</x:v>
+      </x:c>
+      <x:c r="Z11" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA11" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB11" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="30" t="str">
@@ -6241,6 +7251,33 @@
       <x:c r="Q12" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R12" s="47" t="str"/>
+      <x:c r="S12" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-011</x:v>
+      </x:c>
+      <x:c r="T12" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U12" s="47" t="str"/>
+      <x:c r="V12" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-011</x:v>
+      </x:c>
+      <x:c r="W12" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X12" s="47" t="str"/>
+      <x:c r="Y12" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-011</x:v>
+      </x:c>
+      <x:c r="Z12" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA12" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB12" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="30" t="str">
@@ -6294,6 +7331,33 @@
       <x:c r="Q13" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R13" s="47" t="str"/>
+      <x:c r="S13" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-012</x:v>
+      </x:c>
+      <x:c r="T13" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U13" s="47" t="str"/>
+      <x:c r="V13" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-012</x:v>
+      </x:c>
+      <x:c r="W13" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X13" s="47" t="str"/>
+      <x:c r="Y13" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-012</x:v>
+      </x:c>
+      <x:c r="Z13" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA13" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB13" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="30" t="str">
@@ -6347,6 +7411,33 @@
       <x:c r="Q14" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R14" s="47" t="str"/>
+      <x:c r="S14" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-013</x:v>
+      </x:c>
+      <x:c r="T14" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U14" s="47" t="str"/>
+      <x:c r="V14" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-013</x:v>
+      </x:c>
+      <x:c r="W14" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X14" s="47" t="str"/>
+      <x:c r="Y14" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-013</x:v>
+      </x:c>
+      <x:c r="Z14" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA14" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB14" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="30" t="str">
@@ -6400,6 +7491,33 @@
       <x:c r="Q15" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R15" s="47" t="str"/>
+      <x:c r="S15" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-014</x:v>
+      </x:c>
+      <x:c r="T15" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U15" s="47" t="str"/>
+      <x:c r="V15" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-014</x:v>
+      </x:c>
+      <x:c r="W15" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X15" s="47" t="str"/>
+      <x:c r="Y15" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-014</x:v>
+      </x:c>
+      <x:c r="Z15" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA15" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB15" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="30" t="str">
@@ -6453,6 +7571,33 @@
       <x:c r="Q16" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R16" s="47" t="str"/>
+      <x:c r="S16" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-015</x:v>
+      </x:c>
+      <x:c r="T16" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U16" s="47" t="str"/>
+      <x:c r="V16" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-015</x:v>
+      </x:c>
+      <x:c r="W16" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X16" s="47" t="str"/>
+      <x:c r="Y16" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-015</x:v>
+      </x:c>
+      <x:c r="Z16" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA16" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB16" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="30" t="str">
@@ -6506,6 +7651,33 @@
       <x:c r="Q17" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R17" s="47" t="str"/>
+      <x:c r="S17" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-016</x:v>
+      </x:c>
+      <x:c r="T17" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U17" s="47" t="str"/>
+      <x:c r="V17" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-016</x:v>
+      </x:c>
+      <x:c r="W17" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X17" s="47" t="str"/>
+      <x:c r="Y17" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-016</x:v>
+      </x:c>
+      <x:c r="Z17" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA17" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB17" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="30" t="str">
@@ -6559,6 +7731,33 @@
       <x:c r="Q18" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R18" s="47" t="str"/>
+      <x:c r="S18" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-017</x:v>
+      </x:c>
+      <x:c r="T18" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U18" s="47" t="str"/>
+      <x:c r="V18" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-017</x:v>
+      </x:c>
+      <x:c r="W18" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X18" s="47" t="str"/>
+      <x:c r="Y18" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-017</x:v>
+      </x:c>
+      <x:c r="Z18" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA18" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB18" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="30" t="str">
@@ -6612,6 +7811,33 @@
       <x:c r="Q19" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R19" s="47" t="str"/>
+      <x:c r="S19" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-018</x:v>
+      </x:c>
+      <x:c r="T19" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U19" s="47" t="str"/>
+      <x:c r="V19" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-018</x:v>
+      </x:c>
+      <x:c r="W19" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X19" s="47" t="str"/>
+      <x:c r="Y19" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-018</x:v>
+      </x:c>
+      <x:c r="Z19" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA19" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB19" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="30" t="str">
@@ -6665,6 +7891,33 @@
       <x:c r="Q20" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R20" s="47" t="str"/>
+      <x:c r="S20" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-019</x:v>
+      </x:c>
+      <x:c r="T20" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U20" s="47" t="str"/>
+      <x:c r="V20" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-019</x:v>
+      </x:c>
+      <x:c r="W20" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X20" s="47" t="str"/>
+      <x:c r="Y20" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-019</x:v>
+      </x:c>
+      <x:c r="Z20" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA20" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB20" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="30" t="str">
@@ -6718,6 +7971,33 @@
       <x:c r="Q21" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R21" s="47" t="str"/>
+      <x:c r="S21" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-020</x:v>
+      </x:c>
+      <x:c r="T21" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U21" s="47" t="str"/>
+      <x:c r="V21" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-020</x:v>
+      </x:c>
+      <x:c r="W21" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X21" s="47" t="str"/>
+      <x:c r="Y21" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-020</x:v>
+      </x:c>
+      <x:c r="Z21" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA21" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB21" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="30" t="str">
@@ -6771,6 +8051,33 @@
       <x:c r="Q22" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R22" s="47" t="str"/>
+      <x:c r="S22" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-021</x:v>
+      </x:c>
+      <x:c r="T22" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U22" s="47" t="str"/>
+      <x:c r="V22" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-021</x:v>
+      </x:c>
+      <x:c r="W22" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X22" s="47" t="str"/>
+      <x:c r="Y22" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-021</x:v>
+      </x:c>
+      <x:c r="Z22" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA22" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB22" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="30" t="str">
@@ -6824,6 +8131,33 @@
       <x:c r="Q23" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R23" s="47" t="str"/>
+      <x:c r="S23" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-022</x:v>
+      </x:c>
+      <x:c r="T23" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U23" s="47" t="str"/>
+      <x:c r="V23" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-022</x:v>
+      </x:c>
+      <x:c r="W23" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X23" s="47" t="str"/>
+      <x:c r="Y23" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-022</x:v>
+      </x:c>
+      <x:c r="Z23" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA23" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB23" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="30" t="str">
@@ -6877,6 +8211,33 @@
       <x:c r="Q24" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R24" s="47" t="str"/>
+      <x:c r="S24" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-023</x:v>
+      </x:c>
+      <x:c r="T24" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U24" s="47" t="str"/>
+      <x:c r="V24" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-023</x:v>
+      </x:c>
+      <x:c r="W24" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X24" s="47" t="str"/>
+      <x:c r="Y24" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-023</x:v>
+      </x:c>
+      <x:c r="Z24" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA24" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB24" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="30" t="str">
@@ -6930,6 +8291,33 @@
       <x:c r="Q25" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R25" s="47" t="str"/>
+      <x:c r="S25" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-024</x:v>
+      </x:c>
+      <x:c r="T25" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U25" s="47" t="str"/>
+      <x:c r="V25" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-024</x:v>
+      </x:c>
+      <x:c r="W25" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X25" s="47" t="str"/>
+      <x:c r="Y25" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-024</x:v>
+      </x:c>
+      <x:c r="Z25" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA25" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB25" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="30" t="str">
@@ -6983,6 +8371,33 @@
       <x:c r="Q26" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R26" s="47" t="str"/>
+      <x:c r="S26" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-025</x:v>
+      </x:c>
+      <x:c r="T26" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U26" s="47" t="str"/>
+      <x:c r="V26" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-025</x:v>
+      </x:c>
+      <x:c r="W26" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X26" s="47" t="str"/>
+      <x:c r="Y26" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-025</x:v>
+      </x:c>
+      <x:c r="Z26" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA26" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB26" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="30" t="str">
@@ -7036,6 +8451,33 @@
       <x:c r="Q27" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R27" s="47" t="str"/>
+      <x:c r="S27" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-026</x:v>
+      </x:c>
+      <x:c r="T27" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U27" s="47" t="str"/>
+      <x:c r="V27" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-026</x:v>
+      </x:c>
+      <x:c r="W27" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X27" s="47" t="str"/>
+      <x:c r="Y27" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-026</x:v>
+      </x:c>
+      <x:c r="Z27" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA27" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB27" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="30" t="str">
@@ -7089,6 +8531,33 @@
       <x:c r="Q28" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R28" s="47" t="str"/>
+      <x:c r="S28" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-027</x:v>
+      </x:c>
+      <x:c r="T28" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U28" s="47" t="str"/>
+      <x:c r="V28" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-027</x:v>
+      </x:c>
+      <x:c r="W28" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X28" s="47" t="str"/>
+      <x:c r="Y28" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-027</x:v>
+      </x:c>
+      <x:c r="Z28" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA28" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB28" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="30" t="str">
@@ -7142,6 +8611,33 @@
       <x:c r="Q29" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R29" s="47" t="str"/>
+      <x:c r="S29" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-028</x:v>
+      </x:c>
+      <x:c r="T29" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U29" s="47" t="str"/>
+      <x:c r="V29" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-028</x:v>
+      </x:c>
+      <x:c r="W29" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X29" s="47" t="str"/>
+      <x:c r="Y29" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-028</x:v>
+      </x:c>
+      <x:c r="Z29" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA29" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB29" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="30" t="str">
@@ -7195,6 +8691,33 @@
       <x:c r="Q30" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R30" s="47" t="str"/>
+      <x:c r="S30" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-029</x:v>
+      </x:c>
+      <x:c r="T30" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U30" s="47" t="str"/>
+      <x:c r="V30" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-029</x:v>
+      </x:c>
+      <x:c r="W30" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X30" s="47" t="str"/>
+      <x:c r="Y30" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-029</x:v>
+      </x:c>
+      <x:c r="Z30" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA30" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB30" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="30" t="str">
@@ -7248,6 +8771,33 @@
       <x:c r="Q31" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R31" s="47" t="str"/>
+      <x:c r="S31" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-030</x:v>
+      </x:c>
+      <x:c r="T31" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U31" s="47" t="str"/>
+      <x:c r="V31" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-030</x:v>
+      </x:c>
+      <x:c r="W31" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X31" s="47" t="str"/>
+      <x:c r="Y31" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-030</x:v>
+      </x:c>
+      <x:c r="Z31" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA31" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB31" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="30" t="str">
@@ -7301,6 +8851,33 @@
       <x:c r="Q32" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R32" s="47" t="str"/>
+      <x:c r="S32" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-031</x:v>
+      </x:c>
+      <x:c r="T32" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U32" s="47" t="str"/>
+      <x:c r="V32" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-031</x:v>
+      </x:c>
+      <x:c r="W32" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X32" s="47" t="str"/>
+      <x:c r="Y32" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-031</x:v>
+      </x:c>
+      <x:c r="Z32" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA32" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB32" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="30" t="str">
@@ -7354,6 +8931,33 @@
       <x:c r="Q33" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R33" s="47" t="str"/>
+      <x:c r="S33" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-032</x:v>
+      </x:c>
+      <x:c r="T33" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U33" s="47" t="str"/>
+      <x:c r="V33" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-032</x:v>
+      </x:c>
+      <x:c r="W33" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X33" s="47" t="str"/>
+      <x:c r="Y33" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-032</x:v>
+      </x:c>
+      <x:c r="Z33" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA33" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB33" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="30" t="str">
@@ -7407,6 +9011,33 @@
       <x:c r="Q34" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R34" s="47" t="str"/>
+      <x:c r="S34" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-033</x:v>
+      </x:c>
+      <x:c r="T34" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U34" s="47" t="str"/>
+      <x:c r="V34" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-033</x:v>
+      </x:c>
+      <x:c r="W34" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X34" s="47" t="str"/>
+      <x:c r="Y34" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-033</x:v>
+      </x:c>
+      <x:c r="Z34" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA34" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB34" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="30" t="str">
@@ -7460,6 +9091,33 @@
       <x:c r="Q35" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R35" s="47" t="str"/>
+      <x:c r="S35" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-034</x:v>
+      </x:c>
+      <x:c r="T35" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U35" s="47" t="str"/>
+      <x:c r="V35" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-034</x:v>
+      </x:c>
+      <x:c r="W35" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X35" s="47" t="str"/>
+      <x:c r="Y35" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-034</x:v>
+      </x:c>
+      <x:c r="Z35" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA35" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB35" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="30" t="str">
@@ -7513,6 +9171,33 @@
       <x:c r="Q36" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R36" s="47" t="str"/>
+      <x:c r="S36" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-035</x:v>
+      </x:c>
+      <x:c r="T36" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U36" s="47" t="str"/>
+      <x:c r="V36" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-035</x:v>
+      </x:c>
+      <x:c r="W36" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X36" s="47" t="str"/>
+      <x:c r="Y36" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-035</x:v>
+      </x:c>
+      <x:c r="Z36" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA36" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB36" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="30" t="str">
@@ -7566,6 +9251,33 @@
       <x:c r="Q37" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R37" s="47" t="str"/>
+      <x:c r="S37" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-036</x:v>
+      </x:c>
+      <x:c r="T37" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U37" s="47" t="str"/>
+      <x:c r="V37" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-036</x:v>
+      </x:c>
+      <x:c r="W37" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X37" s="47" t="str"/>
+      <x:c r="Y37" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-036</x:v>
+      </x:c>
+      <x:c r="Z37" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA37" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB37" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="30" t="str">
@@ -7619,6 +9331,33 @@
       <x:c r="Q38" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R38" s="47" t="str"/>
+      <x:c r="S38" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-037</x:v>
+      </x:c>
+      <x:c r="T38" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U38" s="47" t="str"/>
+      <x:c r="V38" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-037</x:v>
+      </x:c>
+      <x:c r="W38" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X38" s="47" t="str"/>
+      <x:c r="Y38" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-037</x:v>
+      </x:c>
+      <x:c r="Z38" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA38" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB38" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="30" t="str">
@@ -7672,6 +9411,33 @@
       <x:c r="Q39" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R39" s="47" t="str"/>
+      <x:c r="S39" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-038</x:v>
+      </x:c>
+      <x:c r="T39" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U39" s="47" t="str"/>
+      <x:c r="V39" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-038</x:v>
+      </x:c>
+      <x:c r="W39" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X39" s="47" t="str"/>
+      <x:c r="Y39" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-038</x:v>
+      </x:c>
+      <x:c r="Z39" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA39" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB39" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="30" t="str">
@@ -7725,6 +9491,33 @@
       <x:c r="Q40" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R40" s="47" t="str"/>
+      <x:c r="S40" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-039</x:v>
+      </x:c>
+      <x:c r="T40" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U40" s="47" t="str"/>
+      <x:c r="V40" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-039</x:v>
+      </x:c>
+      <x:c r="W40" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X40" s="47" t="str"/>
+      <x:c r="Y40" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-039</x:v>
+      </x:c>
+      <x:c r="Z40" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA40" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB40" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="30" t="str">
@@ -7778,6 +9571,33 @@
       <x:c r="Q41" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R41" s="47" t="str"/>
+      <x:c r="S41" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-040</x:v>
+      </x:c>
+      <x:c r="T41" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U41" s="47" t="str"/>
+      <x:c r="V41" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-040</x:v>
+      </x:c>
+      <x:c r="W41" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X41" s="47" t="str"/>
+      <x:c r="Y41" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-040</x:v>
+      </x:c>
+      <x:c r="Z41" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA41" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB41" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="30" t="str">
@@ -7831,6 +9651,33 @@
       <x:c r="Q42" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R42" s="47" t="str"/>
+      <x:c r="S42" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-041</x:v>
+      </x:c>
+      <x:c r="T42" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U42" s="47" t="str"/>
+      <x:c r="V42" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-041</x:v>
+      </x:c>
+      <x:c r="W42" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X42" s="47" t="str"/>
+      <x:c r="Y42" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-041</x:v>
+      </x:c>
+      <x:c r="Z42" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA42" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB42" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="30" t="str">
@@ -7884,6 +9731,33 @@
       <x:c r="Q43" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R43" s="47" t="str"/>
+      <x:c r="S43" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-042</x:v>
+      </x:c>
+      <x:c r="T43" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U43" s="47" t="str"/>
+      <x:c r="V43" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-042</x:v>
+      </x:c>
+      <x:c r="W43" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X43" s="47" t="str"/>
+      <x:c r="Y43" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-042</x:v>
+      </x:c>
+      <x:c r="Z43" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA43" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB43" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="30" t="str">
@@ -7937,6 +9811,33 @@
       <x:c r="Q44" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R44" s="47" t="str"/>
+      <x:c r="S44" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-043</x:v>
+      </x:c>
+      <x:c r="T44" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U44" s="47" t="str"/>
+      <x:c r="V44" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-043</x:v>
+      </x:c>
+      <x:c r="W44" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X44" s="47" t="str"/>
+      <x:c r="Y44" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-043</x:v>
+      </x:c>
+      <x:c r="Z44" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA44" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB44" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="30" t="str">
@@ -7990,6 +9891,33 @@
       <x:c r="Q45" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R45" s="47" t="str"/>
+      <x:c r="S45" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-044</x:v>
+      </x:c>
+      <x:c r="T45" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U45" s="47" t="str"/>
+      <x:c r="V45" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-044</x:v>
+      </x:c>
+      <x:c r="W45" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X45" s="47" t="str"/>
+      <x:c r="Y45" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-044</x:v>
+      </x:c>
+      <x:c r="Z45" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA45" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB45" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="30" t="str">
@@ -8043,6 +9971,33 @@
       <x:c r="Q46" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R46" s="47" t="str"/>
+      <x:c r="S46" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-045</x:v>
+      </x:c>
+      <x:c r="T46" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U46" s="47" t="str"/>
+      <x:c r="V46" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-045</x:v>
+      </x:c>
+      <x:c r="W46" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X46" s="47" t="str"/>
+      <x:c r="Y46" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-045</x:v>
+      </x:c>
+      <x:c r="Z46" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA46" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB46" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="30" t="str">
@@ -8096,6 +10051,33 @@
       <x:c r="Q47" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R47" s="47" t="str"/>
+      <x:c r="S47" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-046</x:v>
+      </x:c>
+      <x:c r="T47" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U47" s="47" t="str"/>
+      <x:c r="V47" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-046</x:v>
+      </x:c>
+      <x:c r="W47" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X47" s="47" t="str"/>
+      <x:c r="Y47" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-046</x:v>
+      </x:c>
+      <x:c r="Z47" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA47" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB47" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="30" t="str">
@@ -8149,6 +10131,33 @@
       <x:c r="Q48" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R48" s="47" t="str"/>
+      <x:c r="S48" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-047</x:v>
+      </x:c>
+      <x:c r="T48" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U48" s="47" t="str"/>
+      <x:c r="V48" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-047</x:v>
+      </x:c>
+      <x:c r="W48" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X48" s="47" t="str"/>
+      <x:c r="Y48" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-047</x:v>
+      </x:c>
+      <x:c r="Z48" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA48" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB48" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="30" t="str">
@@ -8202,6 +10211,33 @@
       <x:c r="Q49" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R49" s="47" t="str"/>
+      <x:c r="S49" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-048</x:v>
+      </x:c>
+      <x:c r="T49" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U49" s="47" t="str"/>
+      <x:c r="V49" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-048</x:v>
+      </x:c>
+      <x:c r="W49" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X49" s="47" t="str"/>
+      <x:c r="Y49" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-048</x:v>
+      </x:c>
+      <x:c r="Z49" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA49" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB49" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="30" t="str">
@@ -8255,6 +10291,33 @@
       <x:c r="Q50" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R50" s="47" t="str"/>
+      <x:c r="S50" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-049</x:v>
+      </x:c>
+      <x:c r="T50" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U50" s="47" t="str"/>
+      <x:c r="V50" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-049</x:v>
+      </x:c>
+      <x:c r="W50" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X50" s="47" t="str"/>
+      <x:c r="Y50" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-049</x:v>
+      </x:c>
+      <x:c r="Z50" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA50" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB50" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="30" t="str">
@@ -8308,6 +10371,33 @@
       <x:c r="Q51" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R51" s="47" t="str"/>
+      <x:c r="S51" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-050</x:v>
+      </x:c>
+      <x:c r="T51" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U51" s="47" t="str"/>
+      <x:c r="V51" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-050</x:v>
+      </x:c>
+      <x:c r="W51" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X51" s="47" t="str"/>
+      <x:c r="Y51" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-050</x:v>
+      </x:c>
+      <x:c r="Z51" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA51" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB51" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="30" t="str">
@@ -8361,6 +10451,33 @@
       <x:c r="Q52" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R52" s="47" t="str"/>
+      <x:c r="S52" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-051</x:v>
+      </x:c>
+      <x:c r="T52" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U52" s="47" t="str"/>
+      <x:c r="V52" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-051</x:v>
+      </x:c>
+      <x:c r="W52" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X52" s="47" t="str"/>
+      <x:c r="Y52" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-051</x:v>
+      </x:c>
+      <x:c r="Z52" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA52" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB52" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="30" t="str">
@@ -8414,6 +10531,33 @@
       <x:c r="Q53" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R53" s="47" t="str"/>
+      <x:c r="S53" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-052</x:v>
+      </x:c>
+      <x:c r="T53" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U53" s="47" t="str"/>
+      <x:c r="V53" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-052</x:v>
+      </x:c>
+      <x:c r="W53" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X53" s="47" t="str"/>
+      <x:c r="Y53" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-052</x:v>
+      </x:c>
+      <x:c r="Z53" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA53" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB53" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="30" t="str">
@@ -8467,6 +10611,33 @@
       <x:c r="Q54" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R54" s="47" t="str"/>
+      <x:c r="S54" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-053</x:v>
+      </x:c>
+      <x:c r="T54" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U54" s="47" t="str"/>
+      <x:c r="V54" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-053</x:v>
+      </x:c>
+      <x:c r="W54" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X54" s="47" t="str"/>
+      <x:c r="Y54" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-053</x:v>
+      </x:c>
+      <x:c r="Z54" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA54" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB54" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="30" t="str">
@@ -8520,6 +10691,33 @@
       <x:c r="Q55" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R55" s="47" t="str"/>
+      <x:c r="S55" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-054</x:v>
+      </x:c>
+      <x:c r="T55" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U55" s="47" t="str"/>
+      <x:c r="V55" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-054</x:v>
+      </x:c>
+      <x:c r="W55" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X55" s="47" t="str"/>
+      <x:c r="Y55" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-054</x:v>
+      </x:c>
+      <x:c r="Z55" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA55" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB55" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="30" t="str">
@@ -8573,6 +10771,33 @@
       <x:c r="Q56" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R56" s="47" t="str"/>
+      <x:c r="S56" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-055</x:v>
+      </x:c>
+      <x:c r="T56" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U56" s="47" t="str"/>
+      <x:c r="V56" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-055</x:v>
+      </x:c>
+      <x:c r="W56" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X56" s="47" t="str"/>
+      <x:c r="Y56" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-055</x:v>
+      </x:c>
+      <x:c r="Z56" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA56" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB56" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="30" t="str">
@@ -8626,6 +10851,33 @@
       <x:c r="Q57" s="30" t="str">
         <x:v>Draft - verify follow-up before publishing</x:v>
       </x:c>
+      <x:c r="R57" s="47" t="str"/>
+      <x:c r="S57" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-056</x:v>
+      </x:c>
+      <x:c r="T57" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U57" s="47" t="str"/>
+      <x:c r="V57" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-056</x:v>
+      </x:c>
+      <x:c r="W57" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X57" s="47" t="str"/>
+      <x:c r="Y57" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-056</x:v>
+      </x:c>
+      <x:c r="Z57" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA57" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB57" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="30" t="str">
@@ -8679,11 +10931,43 @@
       <x:c r="Q58" s="30" t="str">
         <x:v>Archive / optional story seed</x:v>
       </x:c>
+      <x:c r="R58" s="47" t="str"/>
+      <x:c r="S58" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 1 for HUM-057</x:v>
+      </x:c>
+      <x:c r="T58" s="47" t="str">
+        <x:v>Before/support context image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="U58" s="47" t="str"/>
+      <x:c r="V58" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 2 for HUM-057</x:v>
+      </x:c>
+      <x:c r="W58" s="47" t="str">
+        <x:v>Support/equipment image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="X58" s="47" t="str"/>
+      <x:c r="Y58" s="47" t="str">
+        <x:v>Anonymized Humanitarians case image 3 for HUM-057</x:v>
+      </x:c>
+      <x:c r="Z58" s="47" t="str">
+        <x:v>Outcome/follow-up image - add only after consent.</x:v>
+      </x:c>
+      <x:c r="AA58" s="47" t="str">
+        <x:v>Pending consent</x:v>
+      </x:c>
+      <x:c r="AB58" s="47" t="str">
+        <x:v>Paste public Google Drive image URLs only after recipient consent and privacy review.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="AA2:AA58">
+      <x:formula1>"Pending consent,Consent received,Do not publish,Review required"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb14cdef3291a4a42"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33790fadb50f4fe5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8750,7 +11034,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe0d20f9e64d4074"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c7d986879924f77"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9001,7 +11285,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ccc27487485430f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra23f4e5d2d074a98"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>